<commit_message>
TradeFinder V4 delivery data integration with historical date matching
</commit_message>
<xml_diff>
--- a/Output/FEATURES.xlsx
+++ b/Output/FEATURES.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:F212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,11 @@
           <t>Volume Ratio</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Delivery %</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +466,9 @@
       <c r="E2" t="n">
         <v>1.007064223020927</v>
       </c>
+      <c r="F2" t="n">
+        <v>47.66</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -480,6 +488,9 @@
       <c r="E3" t="n">
         <v>1.363086982849553</v>
       </c>
+      <c r="F3" t="n">
+        <v>44.16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -499,6 +510,9 @@
       <c r="E4" t="n">
         <v>1.314779319842169</v>
       </c>
+      <c r="F4" t="n">
+        <v>60.79</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -518,6 +532,9 @@
       <c r="E5" t="n">
         <v>0.5732511785235249</v>
       </c>
+      <c r="F5" t="n">
+        <v>55.07</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -537,6 +554,9 @@
       <c r="E6" t="n">
         <v>0.5022414736101887</v>
       </c>
+      <c r="F6" t="n">
+        <v>43.79</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -556,6 +576,9 @@
       <c r="E7" t="n">
         <v>2.924939934367309</v>
       </c>
+      <c r="F7" t="n">
+        <v>47.25</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -575,6 +598,9 @@
       <c r="E8" t="n">
         <v>1.564908322589887</v>
       </c>
+      <c r="F8" t="n">
+        <v>39.05</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -594,6 +620,9 @@
       <c r="E9" t="n">
         <v>7.73744441080335</v>
       </c>
+      <c r="F9" t="n">
+        <v>65.16</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -613,6 +642,9 @@
       <c r="E10" t="n">
         <v>0.6150684162206509</v>
       </c>
+      <c r="F10" t="n">
+        <v>46.85</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -632,6 +664,9 @@
       <c r="E11" t="n">
         <v>1.514841827167246</v>
       </c>
+      <c r="F11" t="n">
+        <v>49.2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -651,6 +686,9 @@
       <c r="E12" t="n">
         <v>1.365947018530817</v>
       </c>
+      <c r="F12" t="n">
+        <v>71.15000000000001</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -670,6 +708,9 @@
       <c r="E13" t="n">
         <v>2.21008361982524</v>
       </c>
+      <c r="F13" t="n">
+        <v>60.05</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -689,6 +730,9 @@
       <c r="E14" t="n">
         <v>2.460246399317628</v>
       </c>
+      <c r="F14" t="n">
+        <v>58.91</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -708,6 +752,9 @@
       <c r="E15" t="n">
         <v>6.337324686486697</v>
       </c>
+      <c r="F15" t="n">
+        <v>58.14</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -727,6 +774,9 @@
       <c r="E16" t="n">
         <v>7.398603026396322</v>
       </c>
+      <c r="F16" t="n">
+        <v>41.82</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -746,6 +796,9 @@
       <c r="E17" t="n">
         <v>0.9621985323800967</v>
       </c>
+      <c r="F17" t="n">
+        <v>63.9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -765,6 +818,9 @@
       <c r="E18" t="n">
         <v>0.1386523160266177</v>
       </c>
+      <c r="F18" t="n">
+        <v>52.46</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -784,6 +840,9 @@
       <c r="E19" t="n">
         <v>0.7430196084176531</v>
       </c>
+      <c r="F19" t="n">
+        <v>71.2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -803,6 +862,9 @@
       <c r="E20" t="n">
         <v>0.417956694143845</v>
       </c>
+      <c r="F20" t="n">
+        <v>51.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -822,6 +884,9 @@
       <c r="E21" t="n">
         <v>4.208099337813025</v>
       </c>
+      <c r="F21" t="n">
+        <v>57.88</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -841,6 +906,9 @@
       <c r="E22" t="n">
         <v>1.579850259144952</v>
       </c>
+      <c r="F22" t="n">
+        <v>62.72</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -860,6 +928,9 @@
       <c r="E23" t="n">
         <v>1.64025406623172</v>
       </c>
+      <c r="F23" t="n">
+        <v>39.75</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -879,6 +950,9 @@
       <c r="E24" t="n">
         <v>6.038321548098084</v>
       </c>
+      <c r="F24" t="n">
+        <v>51.42</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -898,6 +972,9 @@
       <c r="E25" t="n">
         <v>0.4322357112161582</v>
       </c>
+      <c r="F25" t="n">
+        <v>50.96</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -917,6 +994,9 @@
       <c r="E26" t="n">
         <v>3.24571279511922</v>
       </c>
+      <c r="F26" t="n">
+        <v>36.18</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -936,6 +1016,9 @@
       <c r="E27" t="n">
         <v>2.806155669284161</v>
       </c>
+      <c r="F27" t="n">
+        <v>61.9</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -955,6 +1038,9 @@
       <c r="E28" t="n">
         <v>1.225934679845294</v>
       </c>
+      <c r="F28" t="n">
+        <v>53.95</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -974,6 +1060,9 @@
       <c r="E29" t="n">
         <v>0.3841506491646157</v>
       </c>
+      <c r="F29" t="n">
+        <v>59.88</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -993,6 +1082,9 @@
       <c r="E30" t="n">
         <v>0.6082308636428748</v>
       </c>
+      <c r="F30" t="n">
+        <v>66.42</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1012,6 +1104,9 @@
       <c r="E31" t="n">
         <v>9.818966008386399</v>
       </c>
+      <c r="F31" t="n">
+        <v>54.12</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1031,6 +1126,9 @@
       <c r="E32" t="n">
         <v>65.23126611516975</v>
       </c>
+      <c r="F32" t="n">
+        <v>39.53</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1050,6 +1148,9 @@
       <c r="E33" t="n">
         <v>1.833522971441966</v>
       </c>
+      <c r="F33" t="n">
+        <v>55.05</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1069,6 +1170,9 @@
       <c r="E34" t="n">
         <v>5.232967160865206</v>
       </c>
+      <c r="F34" t="n">
+        <v>47.43</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1088,6 +1192,9 @@
       <c r="E35" t="n">
         <v>1.435613792631949</v>
       </c>
+      <c r="F35" t="n">
+        <v>36.28</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1107,6 +1214,9 @@
       <c r="E36" t="n">
         <v>1.293479623263143</v>
       </c>
+      <c r="F36" t="n">
+        <v>57.19</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1126,6 +1236,9 @@
       <c r="E37" t="n">
         <v>0.7322513380474275</v>
       </c>
+      <c r="F37" t="n">
+        <v>66.23999999999999</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1145,6 +1258,9 @@
       <c r="E38" t="n">
         <v>13.40527698558425</v>
       </c>
+      <c r="F38" t="n">
+        <v>56.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1164,6 +1280,9 @@
       <c r="E39" t="n">
         <v>1.090272623093852</v>
       </c>
+      <c r="F39" t="n">
+        <v>46.97</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1183,6 +1302,9 @@
       <c r="E40" t="n">
         <v>4.049593214048521</v>
       </c>
+      <c r="F40" t="n">
+        <v>50.65</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1202,6 +1324,9 @@
       <c r="E41" t="n">
         <v>199.2925330605149</v>
       </c>
+      <c r="F41" t="n">
+        <v>28.18</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1221,6 +1346,9 @@
       <c r="E42" t="n">
         <v>0.4213848302535453</v>
       </c>
+      <c r="F42" t="n">
+        <v>62.92</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1240,6 +1368,9 @@
       <c r="E43" t="n">
         <v>0.813005837272597</v>
       </c>
+      <c r="F43" t="n">
+        <v>43.81</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1259,6 +1390,9 @@
       <c r="E44" t="n">
         <v>3.166558011355497</v>
       </c>
+      <c r="F44" t="n">
+        <v>45.73</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1278,6 +1412,9 @@
       <c r="E45" t="n">
         <v>2.006196608326496</v>
       </c>
+      <c r="F45" t="n">
+        <v>53.84</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1297,6 +1434,9 @@
       <c r="E46" t="n">
         <v>10.10245788894532</v>
       </c>
+      <c r="F46" t="n">
+        <v>60.68</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1316,6 +1456,9 @@
       <c r="E47" t="n">
         <v>0.9574583935617456</v>
       </c>
+      <c r="F47" t="n">
+        <v>51.38</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1335,6 +1478,9 @@
       <c r="E48" t="n">
         <v>0.4015395684390098</v>
       </c>
+      <c r="F48" t="n">
+        <v>52.09</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1354,6 +1500,9 @@
       <c r="E49" t="n">
         <v>1.847381610475186</v>
       </c>
+      <c r="F49" t="n">
+        <v>58.17</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1373,6 +1522,9 @@
       <c r="E50" t="n">
         <v>0.1349905913453399</v>
       </c>
+      <c r="F50" t="n">
+        <v>56.59</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1392,6 +1544,9 @@
       <c r="E51" t="n">
         <v>1.619406489692802</v>
       </c>
+      <c r="F51" t="n">
+        <v>70.34999999999999</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1411,6 +1566,9 @@
       <c r="E52" t="n">
         <v>16.87955823273561</v>
       </c>
+      <c r="F52" t="n">
+        <v>50.09</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1430,6 +1588,9 @@
       <c r="E53" t="n">
         <v>2.134680903361071</v>
       </c>
+      <c r="F53" t="n">
+        <v>68.75</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1449,6 +1610,9 @@
       <c r="E54" t="n">
         <v>0.6439166048104595</v>
       </c>
+      <c r="F54" t="n">
+        <v>60.28</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1468,6 +1632,9 @@
       <c r="E55" t="n">
         <v>0.430662447422224</v>
       </c>
+      <c r="F55" t="n">
+        <v>46.36</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1487,6 +1654,9 @@
       <c r="E56" t="n">
         <v>1.043432824159081</v>
       </c>
+      <c r="F56" t="n">
+        <v>43.98</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1506,6 +1676,9 @@
       <c r="E57" t="n">
         <v>5.106083395189541</v>
       </c>
+      <c r="F57" t="n">
+        <v>48.17</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1525,6 +1698,9 @@
       <c r="E58" t="n">
         <v>4.685022089177117</v>
       </c>
+      <c r="F58" t="n">
+        <v>48.1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1544,6 +1720,9 @@
       <c r="E59" t="n">
         <v>1.512494139938274</v>
       </c>
+      <c r="F59" t="n">
+        <v>55.53</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1563,6 +1742,9 @@
       <c r="E60" t="n">
         <v>0.659162125118829</v>
       </c>
+      <c r="F60" t="n">
+        <v>64.14</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1582,6 +1764,9 @@
       <c r="E61" t="n">
         <v>0.5060260968082197</v>
       </c>
+      <c r="F61" t="n">
+        <v>47.32</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1601,6 +1786,9 @@
       <c r="E62" t="n">
         <v>15.26864313526325</v>
       </c>
+      <c r="F62" t="n">
+        <v>47.53</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1620,6 +1808,9 @@
       <c r="E63" t="n">
         <v>5.064647875402065</v>
       </c>
+      <c r="F63" t="n">
+        <v>57.73</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1639,6 +1830,9 @@
       <c r="E64" t="n">
         <v>6.387167360107305</v>
       </c>
+      <c r="F64" t="n">
+        <v>55.46</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1658,6 +1852,9 @@
       <c r="E65" t="n">
         <v>0.3926640166165306</v>
       </c>
+      <c r="F65" t="n">
+        <v>46.68</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1677,6 +1874,9 @@
       <c r="E66" t="n">
         <v>18.6294438801422</v>
       </c>
+      <c r="F66" t="n">
+        <v>60.53</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1696,6 +1896,9 @@
       <c r="E67" t="n">
         <v>0.3069549165917881</v>
       </c>
+      <c r="F67" t="n">
+        <v>56.71</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1715,6 +1918,9 @@
       <c r="E68" t="n">
         <v>0.1696548911981873</v>
       </c>
+      <c r="F68" t="n">
+        <v>45.14</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1734,6 +1940,9 @@
       <c r="E69" t="n">
         <v>4.549423923376438</v>
       </c>
+      <c r="F69" t="n">
+        <v>43.3</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1753,6 +1962,9 @@
       <c r="E70" t="n">
         <v>1.303097449570913</v>
       </c>
+      <c r="F70" t="n">
+        <v>57.74</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1772,6 +1984,9 @@
       <c r="E71" t="n">
         <v>4.877359895690901</v>
       </c>
+      <c r="F71" t="n">
+        <v>60.44</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1791,6 +2006,9 @@
       <c r="E72" t="n">
         <v>0.500464328502038</v>
       </c>
+      <c r="F72" t="n">
+        <v>60.42</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1810,6 +2028,9 @@
       <c r="E73" t="n">
         <v>1.096391911161464</v>
       </c>
+      <c r="F73" t="n">
+        <v>35.7</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1829,6 +2050,9 @@
       <c r="E74" t="n">
         <v>3.464981654751208</v>
       </c>
+      <c r="F74" t="n">
+        <v>64.31</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1848,6 +2072,9 @@
       <c r="E75" t="n">
         <v>1.023818302275006</v>
       </c>
+      <c r="F75" t="n">
+        <v>40.94</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1867,6 +2094,9 @@
       <c r="E76" t="n">
         <v>0.3535863577763019</v>
       </c>
+      <c r="F76" t="n">
+        <v>60.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1886,6 +2116,9 @@
       <c r="E77" t="n">
         <v>0.4564686942480238</v>
       </c>
+      <c r="F77" t="n">
+        <v>49.07</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1905,6 +2138,9 @@
       <c r="E78" t="n">
         <v>0.3622865146957326</v>
       </c>
+      <c r="F78" t="n">
+        <v>68.34</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1924,6 +2160,9 @@
       <c r="E79" t="n">
         <v>0.7717595486450235</v>
       </c>
+      <c r="F79" t="n">
+        <v>48.92</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1943,6 +2182,9 @@
       <c r="E80" t="n">
         <v>5.946273407691005</v>
       </c>
+      <c r="F80" t="n">
+        <v>51.59</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1962,6 +2204,9 @@
       <c r="E81" t="n">
         <v>2.943718176609238</v>
       </c>
+      <c r="F81" t="n">
+        <v>52.12</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1981,6 +2226,9 @@
       <c r="E82" t="n">
         <v>18.27177257100442</v>
       </c>
+      <c r="F82" t="n">
+        <v>58.7</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2000,6 +2248,9 @@
       <c r="E83" t="n">
         <v>0.262606864736753</v>
       </c>
+      <c r="F83" t="n">
+        <v>46.98</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2019,6 +2270,9 @@
       <c r="E84" t="n">
         <v>7.487065948483546</v>
       </c>
+      <c r="F84" t="n">
+        <v>48.61</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2038,6 +2292,9 @@
       <c r="E85" t="n">
         <v>2.122658010053261</v>
       </c>
+      <c r="F85" t="n">
+        <v>53.24</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2057,6 +2314,9 @@
       <c r="E86" t="n">
         <v>1.733405851597192</v>
       </c>
+      <c r="F86" t="n">
+        <v>50.67</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2076,6 +2336,9 @@
       <c r="E87" t="n">
         <v>0.3935059935409098</v>
       </c>
+      <c r="F87" t="n">
+        <v>39.37</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2095,6 +2358,9 @@
       <c r="E88" t="n">
         <v>0.2549570424919587</v>
       </c>
+      <c r="F88" t="n">
+        <v>54.87</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2114,6 +2380,9 @@
       <c r="E89" t="n">
         <v>7.586272724017137</v>
       </c>
+      <c r="F89" t="n">
+        <v>57.47</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2133,6 +2402,9 @@
       <c r="E90" t="n">
         <v>0.5056663541300412</v>
       </c>
+      <c r="F90" t="n">
+        <v>52.77</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2152,6 +2424,9 @@
       <c r="E91" t="n">
         <v>0.8853507409722493</v>
       </c>
+      <c r="F91" t="n">
+        <v>48.15</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2171,6 +2446,9 @@
       <c r="E92" t="n">
         <v>0.6263323501451993</v>
       </c>
+      <c r="F92" t="n">
+        <v>44.47</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2190,6 +2468,9 @@
       <c r="E93" t="n">
         <v>1.591677410113164</v>
       </c>
+      <c r="F93" t="n">
+        <v>65.14</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2209,6 +2490,9 @@
       <c r="E94" t="n">
         <v>0.6982108905991588</v>
       </c>
+      <c r="F94" t="n">
+        <v>61.08</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2228,6 +2512,9 @@
       <c r="E95" t="n">
         <v>4.126189104191898</v>
       </c>
+      <c r="F95" t="n">
+        <v>51.93</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2247,6 +2534,9 @@
       <c r="E96" t="n">
         <v>8.521357076350093</v>
       </c>
+      <c r="F96" t="n">
+        <v>46.82</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2266,6 +2556,9 @@
       <c r="E97" t="n">
         <v>4.958852192965321</v>
       </c>
+      <c r="F97" t="n">
+        <v>39.55</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2285,6 +2578,9 @@
       <c r="E98" t="n">
         <v>0.08546615163235274</v>
       </c>
+      <c r="F98" t="n">
+        <v>41.6</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2304,6 +2600,9 @@
       <c r="E99" t="n">
         <v>0.1329131180737326</v>
       </c>
+      <c r="F99" t="n">
+        <v>61.23</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2323,6 +2622,9 @@
       <c r="E100" t="n">
         <v>2.224442398848824</v>
       </c>
+      <c r="F100" t="n">
+        <v>32.1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2342,6 +2644,9 @@
       <c r="E101" t="n">
         <v>1.147662160930317</v>
       </c>
+      <c r="F101" t="n">
+        <v>42.18</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2361,6 +2666,9 @@
       <c r="E102" t="n">
         <v>13.70857058444349</v>
       </c>
+      <c r="F102" t="n">
+        <v>56.17</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2380,6 +2688,9 @@
       <c r="E103" t="n">
         <v>4.542216454402209</v>
       </c>
+      <c r="F103" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2399,6 +2710,9 @@
       <c r="E104" t="n">
         <v>0.9075355510411376</v>
       </c>
+      <c r="F104" t="n">
+        <v>50.37</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2418,6 +2732,9 @@
       <c r="E105" t="n">
         <v>0.5928518641507469</v>
       </c>
+      <c r="F105" t="n">
+        <v>65.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2437,6 +2754,9 @@
       <c r="E106" t="n">
         <v>0.4362409006263755</v>
       </c>
+      <c r="F106" t="n">
+        <v>59.59</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2456,6 +2776,9 @@
       <c r="E107" t="n">
         <v>1.66792942857887</v>
       </c>
+      <c r="F107" t="n">
+        <v>64.89</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2475,6 +2798,9 @@
       <c r="E108" t="n">
         <v>1.775672767642041</v>
       </c>
+      <c r="F108" t="n">
+        <v>49.85</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2494,6 +2820,9 @@
       <c r="E109" t="n">
         <v>12.28701931215898</v>
       </c>
+      <c r="F109" t="n">
+        <v>61.41</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2513,6 +2842,9 @@
       <c r="E110" t="n">
         <v>1</v>
       </c>
+      <c r="F110" t="n">
+        <v>56.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2532,6 +2864,9 @@
       <c r="E111" t="n">
         <v>4.188055891966506</v>
       </c>
+      <c r="F111" t="n">
+        <v>53.25</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2551,6 +2886,9 @@
       <c r="E112" t="n">
         <v>8.809582991496399</v>
       </c>
+      <c r="F112" t="n">
+        <v>47.63</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2570,6 +2908,9 @@
       <c r="E113" t="n">
         <v>0.7670478962378404</v>
       </c>
+      <c r="F113" t="n">
+        <v>68.89</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2589,6 +2930,9 @@
       <c r="E114" t="n">
         <v>0.741248567540467</v>
       </c>
+      <c r="F114" t="n">
+        <v>60.8</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2608,6 +2952,9 @@
       <c r="E115" t="n">
         <v>0.8089851838106028</v>
       </c>
+      <c r="F115" t="n">
+        <v>51.01</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2627,6 +2974,9 @@
       <c r="E116" t="n">
         <v>2.123780781602011</v>
       </c>
+      <c r="F116" t="n">
+        <v>63.3</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2646,6 +2996,9 @@
       <c r="E117" t="n">
         <v>0.1457792091521142</v>
       </c>
+      <c r="F117" t="n">
+        <v>49.5</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2665,6 +3018,9 @@
       <c r="E118" t="n">
         <v>0.6912081168366084</v>
       </c>
+      <c r="F118" t="n">
+        <v>53.61</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2684,6 +3040,9 @@
       <c r="E119" t="n">
         <v>4.100850441457983</v>
       </c>
+      <c r="F119" t="n">
+        <v>59.92</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2703,6 +3062,9 @@
       <c r="E120" t="n">
         <v>0.3438000546939095</v>
       </c>
+      <c r="F120" t="n">
+        <v>49.74</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2722,6 +3084,9 @@
       <c r="E121" t="n">
         <v>0.5554402534151137</v>
       </c>
+      <c r="F121" t="n">
+        <v>62.33</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2741,6 +3106,9 @@
       <c r="E122" t="n">
         <v>0.6573772479847899</v>
       </c>
+      <c r="F122" t="n">
+        <v>45.86</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2760,6 +3128,9 @@
       <c r="E123" t="n">
         <v>0.1896857216340457</v>
       </c>
+      <c r="F123" t="n">
+        <v>57.93</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2779,6 +3150,9 @@
       <c r="E124" t="n">
         <v>0.2744030876014116</v>
       </c>
+      <c r="F124" t="n">
+        <v>54.11</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2798,6 +3172,9 @@
       <c r="E125" t="n">
         <v>0.3066672038389915</v>
       </c>
+      <c r="F125" t="n">
+        <v>56.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2817,6 +3194,9 @@
       <c r="E126" t="n">
         <v>1.418633042934719</v>
       </c>
+      <c r="F126" t="n">
+        <v>56.25</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2836,6 +3216,9 @@
       <c r="E127" t="n">
         <v>0.8543038083890039</v>
       </c>
+      <c r="F127" t="n">
+        <v>48.06</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2855,6 +3238,9 @@
       <c r="E128" t="n">
         <v>0.0374873031995937</v>
       </c>
+      <c r="F128" t="n">
+        <v>53.15</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2874,6 +3260,9 @@
       <c r="E129" t="n">
         <v>1.290540232579339</v>
       </c>
+      <c r="F129" t="n">
+        <v>41.38</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2893,6 +3282,9 @@
       <c r="E130" t="n">
         <v>1.814661304710187</v>
       </c>
+      <c r="F130" t="n">
+        <v>41.76</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2912,6 +3304,9 @@
       <c r="E131" t="n">
         <v>0.4397976325350627</v>
       </c>
+      <c r="F131" t="n">
+        <v>62.62</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2931,6 +3326,9 @@
       <c r="E132" t="n">
         <v>0.4466445449336511</v>
       </c>
+      <c r="F132" t="n">
+        <v>42.1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2950,6 +3348,9 @@
       <c r="E133" t="n">
         <v>1.460141813493769</v>
       </c>
+      <c r="F133" t="n">
+        <v>40.5</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2969,6 +3370,9 @@
       <c r="E134" t="n">
         <v>3.718427696605071</v>
       </c>
+      <c r="F134" t="n">
+        <v>33.56</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2988,6 +3392,9 @@
       <c r="E135" t="n">
         <v>0.08858500670651509</v>
       </c>
+      <c r="F135" t="n">
+        <v>26.29</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3007,6 +3414,9 @@
       <c r="E136" t="n">
         <v>0.3379648168405152</v>
       </c>
+      <c r="F136" t="n">
+        <v>41.2</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3026,6 +3436,9 @@
       <c r="E137" t="n">
         <v>0.1990776913961272</v>
       </c>
+      <c r="F137" t="n">
+        <v>55.1</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3045,6 +3458,9 @@
       <c r="E138" t="n">
         <v>0.1834944036410517</v>
       </c>
+      <c r="F138" t="n">
+        <v>40.4</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3064,6 +3480,9 @@
       <c r="E139" t="n">
         <v>2.887700462944876</v>
       </c>
+      <c r="F139" t="n">
+        <v>63.33</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3083,6 +3502,9 @@
       <c r="E140" t="n">
         <v>0.7647567748824732</v>
       </c>
+      <c r="F140" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3102,6 +3524,9 @@
       <c r="E141" t="n">
         <v>0.1544187307106301</v>
       </c>
+      <c r="F141" t="n">
+        <v>57.23</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3121,6 +3546,9 @@
       <c r="E142" t="n">
         <v>1.008430756859528</v>
       </c>
+      <c r="F142" t="n">
+        <v>48.01</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3140,6 +3568,9 @@
       <c r="E143" t="n">
         <v>49.23852282494042</v>
       </c>
+      <c r="F143" t="n">
+        <v>44.37</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3159,6 +3590,9 @@
       <c r="E144" t="n">
         <v>0.2351992746545819</v>
       </c>
+      <c r="F144" t="n">
+        <v>64.53</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3178,6 +3612,9 @@
       <c r="E145" t="n">
         <v>0.4978281146228073</v>
       </c>
+      <c r="F145" t="n">
+        <v>37.69</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3197,6 +3634,9 @@
       <c r="E146" t="n">
         <v>0.9854410022007787</v>
       </c>
+      <c r="F146" t="n">
+        <v>47.23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3216,6 +3656,9 @@
       <c r="E147" t="n">
         <v>0.9955748394994205</v>
       </c>
+      <c r="F147" t="n">
+        <v>51.96</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3235,6 +3678,9 @@
       <c r="E148" t="n">
         <v>1.342686642965973</v>
       </c>
+      <c r="F148" t="n">
+        <v>39.21</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3254,6 +3700,9 @@
       <c r="E149" t="n">
         <v>10.42461315453634</v>
       </c>
+      <c r="F149" t="n">
+        <v>51.85</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3273,6 +3722,9 @@
       <c r="E150" t="n">
         <v>0.4333556341237905</v>
       </c>
+      <c r="F150" t="n">
+        <v>60.22</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3292,6 +3744,9 @@
       <c r="E151" t="n">
         <v>4.517619659204855</v>
       </c>
+      <c r="F151" t="n">
+        <v>49.4</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3311,6 +3766,9 @@
       <c r="E152" t="n">
         <v>1.774933341797867</v>
       </c>
+      <c r="F152" t="n">
+        <v>50.04</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3330,6 +3788,9 @@
       <c r="E153" t="n">
         <v>0.4827172943443893</v>
       </c>
+      <c r="F153" t="n">
+        <v>42.81</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3349,6 +3810,9 @@
       <c r="E154" t="n">
         <v>0.3460069376619656</v>
       </c>
+      <c r="F154" t="n">
+        <v>41.78</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3368,6 +3832,9 @@
       <c r="E155" t="n">
         <v>1.146812858928781</v>
       </c>
+      <c r="F155" t="n">
+        <v>61.31</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3387,6 +3854,9 @@
       <c r="E156" t="n">
         <v>0.5658288406193435</v>
       </c>
+      <c r="F156" t="n">
+        <v>39.88</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3406,6 +3876,9 @@
       <c r="E157" t="n">
         <v>0.3269975485408446</v>
       </c>
+      <c r="F157" t="n">
+        <v>48.63</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3425,6 +3898,9 @@
       <c r="E158" t="n">
         <v>0.192874164941204</v>
       </c>
+      <c r="F158" t="n">
+        <v>45.7</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3444,6 +3920,9 @@
       <c r="E159" t="n">
         <v>0.2631208409839695</v>
       </c>
+      <c r="F159" t="n">
+        <v>62.55</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3463,6 +3942,9 @@
       <c r="E160" t="n">
         <v>1.856479356304775</v>
       </c>
+      <c r="F160" t="n">
+        <v>40.34</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3482,6 +3964,9 @@
       <c r="E161" t="n">
         <v>9.821464266645831</v>
       </c>
+      <c r="F161" t="n">
+        <v>48.04</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3501,6 +3986,9 @@
       <c r="E162" t="n">
         <v>0.2982987101353023</v>
       </c>
+      <c r="F162" t="n">
+        <v>49.84</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3520,6 +4008,9 @@
       <c r="E163" t="n">
         <v>0.0125942493260929</v>
       </c>
+      <c r="F163" t="n">
+        <v>52.17</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3539,6 +4030,9 @@
       <c r="E164" t="n">
         <v>1.332597570027738</v>
       </c>
+      <c r="F164" t="n">
+        <v>52.09</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3558,6 +4052,9 @@
       <c r="E165" t="n">
         <v>4.399241935903947</v>
       </c>
+      <c r="F165" t="n">
+        <v>53.81</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3577,6 +4074,9 @@
       <c r="E166" t="n">
         <v>0.1950810479092602</v>
       </c>
+      <c r="F166" t="n">
+        <v>62.51</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3596,6 +4096,9 @@
       <c r="E167" t="n">
         <v>0.3179942148168405</v>
       </c>
+      <c r="F167" t="n">
+        <v>53.97</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3615,6 +4118,9 @@
       <c r="E168" t="n">
         <v>7.545763826490083</v>
       </c>
+      <c r="F168" t="n">
+        <v>50.98</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3634,6 +4140,9 @@
       <c r="E169" t="n">
         <v>0.166015141748382</v>
       </c>
+      <c r="F169" t="n">
+        <v>39.86</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3653,6 +4162,9 @@
       <c r="E170" t="n">
         <v>8.692677608704145</v>
       </c>
+      <c r="F170" t="n">
+        <v>52.89</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3672,6 +4184,9 @@
       <c r="E171" t="n">
         <v>5.846099315023896</v>
       </c>
+      <c r="F171" t="n">
+        <v>56.16</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3691,6 +4206,9 @@
       <c r="E172" t="n">
         <v>0.5851080367490982</v>
       </c>
+      <c r="F172" t="n">
+        <v>56.23</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3710,6 +4228,9 @@
       <c r="E173" t="n">
         <v>0.3479244800823013</v>
       </c>
+      <c r="F173" t="n">
+        <v>55.02</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3729,6 +4250,9 @@
       <c r="E174" t="n">
         <v>0.5749078668073081</v>
       </c>
+      <c r="F174" t="n">
+        <v>56.28</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3748,6 +4272,9 @@
       <c r="E175" t="n">
         <v>1.025657303590265</v>
       </c>
+      <c r="F175" t="n">
+        <v>41.96</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3767,6 +4294,9 @@
       <c r="E176" t="n">
         <v>2.505892617624461</v>
       </c>
+      <c r="F176" t="n">
+        <v>28.35</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3786,6 +4316,9 @@
       <c r="E177" t="n">
         <v>6.972716529280775</v>
       </c>
+      <c r="F177" t="n">
+        <v>42.8</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3805,6 +4338,9 @@
       <c r="E178" t="n">
         <v>2.786952165618367</v>
       </c>
+      <c r="F178" t="n">
+        <v>55.33</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3824,6 +4360,9 @@
       <c r="E179" t="n">
         <v>0.0178719674180568</v>
       </c>
+      <c r="F179" t="n">
+        <v>48.89</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3843,6 +4382,9 @@
       <c r="E180" t="n">
         <v>0.1301442389082054</v>
       </c>
+      <c r="F180" t="n">
+        <v>39.09</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3862,6 +4404,9 @@
       <c r="E181" t="n">
         <v>1.544058304358584</v>
       </c>
+      <c r="F181" t="n">
+        <v>46.89</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3881,6 +4426,9 @@
       <c r="E182" t="n">
         <v>9.23683724329674</v>
       </c>
+      <c r="F182" t="n">
+        <v>33.78</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3900,6 +4448,9 @@
       <c r="E183" t="n">
         <v>0.7024065320154705</v>
       </c>
+      <c r="F183" t="n">
+        <v>43.41</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3919,6 +4470,9 @@
       <c r="E184" t="n">
         <v>1.934764083681682</v>
       </c>
+      <c r="F184" t="n">
+        <v>47.14</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3938,6 +4492,9 @@
       <c r="E185" t="n">
         <v>0.3146779896081572</v>
       </c>
+      <c r="F185" t="n">
+        <v>45.96</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3957,6 +4514,9 @@
       <c r="E186" t="n">
         <v>0.1999058320636533</v>
       </c>
+      <c r="F186" t="n">
+        <v>61.36</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3976,6 +4536,9 @@
       <c r="E187" t="n">
         <v>0.1239264692476983</v>
       </c>
+      <c r="F187" t="n">
+        <v>37.86</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3995,6 +4558,9 @@
       <c r="E188" t="n">
         <v>7.166058685262596</v>
       </c>
+      <c r="F188" t="n">
+        <v>43.06</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4014,6 +4580,9 @@
       <c r="E189" t="n">
         <v>0.2236407098488104</v>
       </c>
+      <c r="F189" t="n">
+        <v>37.16</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4033,6 +4602,9 @@
       <c r="E190" t="n">
         <v>0.8702700348999232</v>
       </c>
+      <c r="F190" t="n">
+        <v>42.44</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4052,6 +4624,9 @@
       <c r="E191" t="n">
         <v>0.1288607226107226</v>
       </c>
+      <c r="F191" t="n">
+        <v>46.02</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4071,6 +4646,9 @@
       <c r="E192" t="n">
         <v>10.92469454428253</v>
       </c>
+      <c r="F192" t="n">
+        <v>48.83</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4090,6 +4668,9 @@
       <c r="E193" t="n">
         <v>0.1245698551913636</v>
       </c>
+      <c r="F193" t="n">
+        <v>33.58</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4109,6 +4690,9 @@
       <c r="E194" t="n">
         <v>0.1841687176882708</v>
       </c>
+      <c r="F194" t="n">
+        <v>41.68</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4128,6 +4712,9 @@
       <c r="E195" t="n">
         <v>0.6156059954942636</v>
       </c>
+      <c r="F195" t="n">
+        <v>49.78</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4147,6 +4734,9 @@
       <c r="E196" t="n">
         <v>0.4145061758539412</v>
       </c>
+      <c r="F196" t="n">
+        <v>29.56</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4166,6 +4756,9 @@
       <c r="E197" t="n">
         <v>1.650736251644073</v>
       </c>
+      <c r="F197" t="n">
+        <v>40.44</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4185,6 +4778,9 @@
       <c r="E198" t="n">
         <v>0.12276218892839</v>
       </c>
+      <c r="F198" t="n">
+        <v>58.72</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4204,6 +4800,9 @@
       <c r="E199" t="n">
         <v>0.1753782181505645</v>
       </c>
+      <c r="F199" t="n">
+        <v>41.75</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4223,6 +4822,9 @@
       <c r="E200" t="n">
         <v>1.174180161086586</v>
       </c>
+      <c r="F200" t="n">
+        <v>28.96</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4242,6 +4844,9 @@
       <c r="E201" t="n">
         <v>0.2234974638955086</v>
       </c>
+      <c r="F201" t="n">
+        <v>25.8</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4261,6 +4866,9 @@
       <c r="E202" t="n">
         <v>0.01336297547889727</v>
       </c>
+      <c r="F202" t="n">
+        <v>40.08</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4280,6 +4888,9 @@
       <c r="E203" t="n">
         <v>0.1497555052024326</v>
       </c>
+      <c r="F203" t="n">
+        <v>50.85</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4299,6 +4910,9 @@
       <c r="E204" t="n">
         <v>0.5291717128309307</v>
       </c>
+      <c r="F204" t="n">
+        <v>41.05</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4318,6 +4932,9 @@
       <c r="E205" t="n">
         <v>0.1075598051855035</v>
       </c>
+      <c r="F205" t="n">
+        <v>44.46</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4337,6 +4954,9 @@
       <c r="E206" t="n">
         <v>0.2813118562071076</v>
       </c>
+      <c r="F206" t="n">
+        <v>58.22</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4356,6 +4976,9 @@
       <c r="E207" t="n">
         <v>1.855473785990546</v>
       </c>
+      <c r="F207" t="n">
+        <v>39.41</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4375,6 +4998,9 @@
       <c r="E208" t="n">
         <v>0.06501209451628447</v>
       </c>
+      <c r="F208" t="n">
+        <v>24.41</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4394,6 +5020,9 @@
       <c r="E209" t="n">
         <v>0.6160129442252348</v>
       </c>
+      <c r="F209" t="n">
+        <v>40.82</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -4413,6 +5042,9 @@
       <c r="E210" t="n">
         <v>0.6186084632313683</v>
       </c>
+      <c r="F210" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4431,6 +5063,9 @@
       </c>
       <c r="E211" t="n">
         <v>0.05731954265473819</v>
+      </c>
+      <c r="F211" t="n">
+        <v>40.79</v>
       </c>
     </row>
     <row r="212">
@@ -4448,6 +5083,9 @@
       <c r="D212" t="inlineStr"/>
       <c r="E212" t="n">
         <v>27.35854584196065</v>
+      </c>
+      <c r="F212" t="n">
+        <v>53.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>